<commit_message>
change dashboard and add database
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/serena/Desktop/Hunter CRM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA89F9A3-C2B0-034D-B9C0-AEE4D62D508E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19A0F2A-A6A4-3A40-A082-00F2B9EE729B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
   <si>
     <t>date</t>
   </si>
@@ -139,6 +139,15 @@
   </si>
   <si>
     <t>SMS #1 What to Expect (EOI &amp; Build)</t>
+  </si>
+  <si>
+    <t>EDM #3: What does 360kW of power mean? (Reservation)</t>
+  </si>
+  <si>
+    <t>EDM #3: What does 360kW of power mean? (Build)</t>
+  </si>
+  <si>
+    <t>EDM #3: Hunter Pro vs Hunter X (EOI)</t>
   </si>
 </sst>
 </file>
@@ -207,12 +216,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -224,6 +232,10 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,12 +538,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="3" max="3" width="42.1640625" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
     <col min="5" max="8" width="14" customWidth="1"/>
     <col min="9" max="12" width="17" customWidth="1"/>
@@ -546,7 +558,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -586,56 +598,56 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
-        <v>46169</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="2" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="7">
+        <v>46170</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="8">
         <v>68</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
+      <c r="E2" s="8">
+        <v>0</v>
+      </c>
+      <c r="F2" s="8">
         <v>68</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="8">
         <v>68</v>
       </c>
-      <c r="H2">
-        <v>44</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0.64700000000000002</v>
-      </c>
-      <c r="J2">
-        <v>18</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0.26500000000000001</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2" s="7">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2" s="7">
+      <c r="H2" s="8">
+        <v>47</v>
+      </c>
+      <c r="I2" s="9">
+        <v>0.69099999999999995</v>
+      </c>
+      <c r="J2" s="8">
+        <v>19</v>
+      </c>
+      <c r="K2" s="9">
+        <v>0.27900000000000003</v>
+      </c>
+      <c r="L2" s="8">
+        <v>2</v>
+      </c>
+      <c r="M2" s="9">
+        <v>2.9399999999999999E-2</v>
+      </c>
+      <c r="N2" s="8">
+        <v>0</v>
+      </c>
+      <c r="O2" s="10">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
-        <v>46169</v>
+      <c r="A3" s="7">
+        <v>46170</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -656,33 +668,33 @@
         <v>102</v>
       </c>
       <c r="H3">
-        <v>45</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0.30399999999999999</v>
+        <v>32</v>
+      </c>
+      <c r="I3" s="5">
+        <v>0.314</v>
       </c>
       <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3" s="6">
-        <v>0.11799999999999999</v>
+        <v>13</v>
+      </c>
+      <c r="K3" s="5">
+        <v>0.127</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
-      <c r="M3" s="7">
+      <c r="M3" s="6">
         <v>0</v>
       </c>
       <c r="N3">
         <v>0</v>
       </c>
-      <c r="O3" s="7">
+      <c r="O3" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
-        <v>46169</v>
+      <c r="A4" s="7">
+        <v>46170</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
@@ -703,33 +715,33 @@
         <v>866</v>
       </c>
       <c r="H4">
-        <v>290</v>
-      </c>
-      <c r="I4" s="6">
-        <v>0.33500000000000002</v>
+        <v>294</v>
+      </c>
+      <c r="I4" s="5">
+        <v>0.33900000000000002</v>
       </c>
       <c r="J4">
-        <v>79</v>
-      </c>
-      <c r="K4" s="6">
-        <v>9.0999999999999998E-2</v>
+        <v>83</v>
+      </c>
+      <c r="K4" s="5">
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="L4">
         <v>6</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="5">
         <v>6.8999999999999999E-3</v>
       </c>
       <c r="N4">
         <v>1</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="5">
         <v>1.1999999999999999E-3</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
-        <v>46169</v>
+      <c r="A5" s="7">
+        <v>46170</v>
       </c>
       <c r="B5" t="s">
         <v>30</v>
@@ -740,6 +752,9 @@
       <c r="D5">
         <v>68</v>
       </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
       <c r="F5">
         <v>68</v>
       </c>
@@ -749,19 +764,19 @@
       <c r="J5">
         <v>38</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="5">
         <v>0.57599999999999996</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
-      <c r="M5" s="7">
+      <c r="M5" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
-        <v>46169</v>
+      <c r="A6" s="7">
+        <v>46170</v>
       </c>
       <c r="B6" t="s">
         <v>32</v>
@@ -772,6 +787,9 @@
       <c r="D6">
         <v>752</v>
       </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
       <c r="F6">
         <v>752</v>
       </c>
@@ -781,18 +799,94 @@
       <c r="J6">
         <v>302</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="5">
         <v>0.41199999999999998</v>
       </c>
       <c r="L6">
         <v>25</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="5">
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
+    <row r="7" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="7">
+        <v>46177</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="8">
+        <v>69</v>
+      </c>
+      <c r="E7" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" s="7">
+        <v>46177</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8">
+        <v>110</v>
+      </c>
+      <c r="E8" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" s="7">
+        <v>46177</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9">
+        <v>890</v>
+      </c>
+      <c r="E9" s="8">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" s="7">
+        <v>46177</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" s="7">
+        <v>46177</v>
+      </c>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -811,58 +905,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="4" t="s">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>